<commit_message>
Fix datasets processing and add splits to results
Change -pH to pH in my datasets and recovered the original file
containing distribution of events in the datasets in order to
recreate datasets compatible with already trained models

Add data splits to the visualization functionality of results
Refactore code of the results and fix a few insignificant glitches
</commit_message>
<xml_diff>
--- a/training/training_log.xlsx
+++ b/training/training_log.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Work\Data analysis in Python\ML_paper1\results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Work\Data analysis in Python\ML_paper1\imputation-research\training\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C44C193-D559-4FD3-959A-11890AA8D616}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51A7BD22-E519-496B-AC87-7EC5AD00286B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{67663D26-D449-4C21-9C49-EF5664B29A7E}"/>
+    <workbookView xWindow="38280" yWindow="2505" windowWidth="29040" windowHeight="15840" xr2:uid="{67663D26-D449-4C21-9C49-EF5664B29A7E}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="12">
   <si>
     <t>5 min</t>
   </si>
@@ -220,7 +220,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -251,35 +251,41 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -660,12 +666,12 @@
       <c r="V1" s="1"/>
     </row>
     <row r="2" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
@@ -733,8 +739,8 @@
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="21"/>
-      <c r="I4" s="17" t="s">
+      <c r="H4" s="20"/>
+      <c r="I4" s="16" t="s">
         <v>10</v>
       </c>
       <c r="J4" s="1"/>
@@ -767,10 +773,10 @@
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
-      <c r="H5" s="18" t="s">
-        <v>6</v>
-      </c>
-      <c r="I5" s="17" t="s">
+      <c r="H5" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="I5" s="16" t="s">
         <v>11</v>
       </c>
       <c r="J5" s="1"/>
@@ -820,12 +826,12 @@
       <c r="V6" s="1"/>
     </row>
     <row r="9" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="12"/>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12"/>
+      <c r="B9" s="21"/>
+      <c r="C9" s="21"/>
+      <c r="D9" s="21"/>
     </row>
     <row r="10" spans="1:22" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
@@ -848,32 +854,36 @@
       <c r="B11" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="19"/>
-      <c r="D11" s="20"/>
+      <c r="C11" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="B12" s="13"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="14"/>
+      <c r="B12" s="18"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="19"/>
     </row>
     <row r="13" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="16"/>
+      <c r="B13" s="22"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="23"/>
     </row>
     <row r="16" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="12" t="s">
+      <c r="A16" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="B16" s="12"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
+      <c r="B16" s="21"/>
+      <c r="C16" s="21"/>
+      <c r="D16" s="21"/>
     </row>
     <row r="17" spans="1:4" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="8" t="s">
@@ -893,25 +903,25 @@
       <c r="A18" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="14"/>
+      <c r="B18" s="12"/>
+      <c r="C18" s="12"/>
+      <c r="D18" s="13"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="B19" s="13"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="14"/>
+      <c r="B19" s="12"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="13"/>
     </row>
     <row r="20" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="B20" s="15"/>
-      <c r="C20" s="15"/>
-      <c r="D20" s="16"/>
+      <c r="B20" s="14"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>